<commit_message>
adding and update student data is completed
</commit_message>
<xml_diff>
--- a/uploads/admissions_template.xlsx
+++ b/uploads/admissions_template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:H2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -422,16 +422,7 @@
         <v>admissionDate</v>
       </c>
       <c r="H1" t="str">
-        <v>admissionMonth</v>
-      </c>
-      <c r="I1" t="str">
-        <v>admissionYear</v>
-      </c>
-      <c r="J1" t="str">
         <v>batchNumber</v>
-      </c>
-      <c r="K1" t="str">
-        <v>status</v>
       </c>
     </row>
     <row r="2">
@@ -459,19 +450,10 @@
       <c r="H2" t="str">
         <v/>
       </c>
-      <c r="I2" t="str">
-        <v/>
-      </c>
-      <c r="J2" t="str">
-        <v/>
-      </c>
-      <c r="K2" t="str">
-        <v/>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>